<commit_message>
feat(s8-np): rerun new pairs with --no-rerank; holdout 1.00/1.00/0.75
The pruner runs with enable_reranker=False; run_pair default enabled
the cross-encoder reranker, which collapsed masked scores into a tight
band and drove holdout accuracy to 0.00. Rerunning all three s8-np
pairs with --no-rerank produces prune-consistent scoring:

  csa_aicm__owasp_agentic: 110 mappings (D=53 R=57) holdout=1.00
  mitre_atlas__owasp_llm:   94 mappings (D=41 R=53) holdout=1.00
  nist_rmf__owasp_agentic:  30 mappings (D=13 R=17) holdout=0.75

All three clear the 0.50 gate. Cross-pair validation refresh shows
the new pairs at MRR 0.57 / 0.71 / 0.72 and Recall@5 0.92 / 0.95 / 1.00,
each above or at the session9 cohort median. Graph grows to 6001 edges
(test_graph count pinned accordingly).

Edges merged into data/processed/edges.json. 89/89 mapping_engine
tests pass including test_s8_frozen_tier_acc_non_inferior.
</commit_message>
<xml_diff>
--- a/mapping_engine/output/results/mitre_atlas__owasp_llm.xlsx
+++ b/mapping_engine/output/results/mitre_atlas__owasp_llm.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-04-07T17:32:26.553105+00:00</t>
+          <t>2026-04-08T12:29:34.799840+00:00</t>
         </is>
       </c>
     </row>
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>81</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7">

</xml_diff>